<commit_message>
Update venue for 7 published papers (arxiv -> formal venues)
- ID 0: arxiv -> NAACL 2025 Workshop
- ID 3: arxiv -> ASE 2025
- ID 5: arxiv -> Automated Software Engineering (journal)
- ID 43: arxiv -> IEEE Transactions on Software Engineering
- ID 45: arxiv -> ACM ESEC/FSE 2025
- ID 53: arxiv -> ASE 2023
- ID 60: arxiv -> Empirical Software Engineering (journal)

Detected via CrossRef API by matching titles and DOIs.
</commit_message>
<xml_diff>
--- a/metadata_manager/output/apr_literature_metadata.xlsx
+++ b/metadata_manager/output/apr_literature_metadata.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,7 +514,6 @@
           <t>Towards Effectively Leveraging Execution Traces for Program Repair with Code LLMs</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>['Mirazul Haque', 'Petr Babkin', 'Farima Farmahinifarahani', 'Manuela Veloso']</t>
@@ -525,10 +524,9 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>arxiv</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>NAACL 2025 Workshop</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>['Java', ' Python']</t>
@@ -556,12 +554,12 @@
   author={Haque, Mirazul and Babkin, Petr and Farmahinifarahani, Farima and Veloso, Manuela},
   journal={arXiv preprint arXiv:2505.04441},
   year={2025}
-}</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+,
+  url          = {https://doi.org/10.18653/v1/2025.knowledgenlp-1.17},
+  doi          = {10.18653/v1/2025.knowledgenlp-1.17},
+}</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -615,7 +613,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>-</t>
@@ -659,7 +656,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>['Python']</t>
@@ -730,10 +726,9 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>arxiv</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>ASE 2025</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>['JavaScript']</t>
@@ -761,6 +756,9 @@
   author={Huang, Kai and Zhang, Jian and Xie, Xiaofei and Chen, Chunyang},
   journal={arXiv preprint arXiv:2506.16136},
   year={2025}
+,
+  url          = {https://doi.org/10.1109/ase63991.2025.00100},
+  doi          = {10.1109/ase63991.2025.00100},
 }</t>
         </is>
       </c>
@@ -882,7 +880,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>arxiv</t>
+          <t>Automated Software Engineering</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -917,6 +915,9 @@
   author={Gharibi, Reza and Sadreddini, Mohammad Hadi and Fakhrahmad, Seyed Mostafa},
   journal={arXiv preprint arXiv:2501.16044},
   year={2025}
+,
+  url          = {https://doi.org/10.1007/s10515-026-00611-2},
+  doi          = {10.1007/s10515-026-00611-2},
 }</t>
         </is>
       </c>
@@ -1026,7 +1027,6 @@
           <t>Comprehensive Fine-Tuning Large Language Models of Code for Automated Program Repair</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>['Kai Huang', 'Jian Zhang', 'Xinlei Bao', 'Xu Wang', 'Yang Liu']</t>
@@ -1076,9 +1076,6 @@
 }</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -1089,7 +1086,6 @@
           <t>Bug Fixing with Broader Context: Enhancing LLM-Based Program Repair via Layered Knowledge Injection</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>['Ramtin Ehsani', 'Esteban Parra', 'Sonia Haiduc', 'Preetha Chatterjee']</t>
@@ -1103,7 +1099,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>['Python']</t>
@@ -1134,9 +1129,6 @@
 }</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1165,7 +1157,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>['C']</t>
@@ -1196,8 +1187,6 @@
 }</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -1231,7 +1220,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>['Java', 'Python']</t>
@@ -1359,7 +1347,6 @@
 }</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>llm-based</t>
@@ -1449,9 +1436,6 @@
 }</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1606,7 +1590,6 @@
 }</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -1965,9 +1948,6 @@
 }</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -2088,7 +2068,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>['Java']</t>
@@ -2122,7 +2101,6 @@
 }</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>llm-based</t>
@@ -2276,7 +2254,6 @@
 }</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -2368,9 +2345,6 @@
 }</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -2381,7 +2355,6 @@
           <t>Poster: Repairing Bugs with the Introduction of New Variables: A Multi-Agent Large Language Model</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>['Elisa Zhang', 'Shiyu Sun', 'Yunlong Xing', 'Kun Sun']</t>
@@ -2395,7 +2368,6 @@
           <t>CCS</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>['Java']</t>
@@ -2427,9 +2399,6 @@
 }</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -3268,7 +3237,6 @@
           <t>Exploring and Lifting the Robustness of LLM-powered Automated Program Repair with Metamorphic Testing</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>['Pengyu Xue', 'Linhao Wu', 'Zhen Yang', 'Zhongxing Yu', 'Zhi Jin', 'Ge Li', 'Yan Xiao', 'Shuo Liu', 'Xinyi Li', 'Hongyi Lin', 'others']</t>
@@ -3282,7 +3250,6 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>['Java', ' Python']</t>
@@ -3313,9 +3280,6 @@
 }</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -3631,7 +3595,6 @@
 }</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>llm-based</t>
@@ -3896,7 +3859,6 @@
 </t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>learning-based, llm-based</t>
@@ -4011,7 +3973,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>arxiv</t>
+          <t>IEEE Transactions on Software Engineering</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4194,7 +4156,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>arxiv</t>
+          <t>ACM ESEC/FSE 2025</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4286,7 +4248,6 @@
           <t>EMSE</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>['']</t>
@@ -4332,8 +4293,6 @@
 }</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -4504,7 +4463,6 @@
 }</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -4863,7 +4821,6 @@
 }</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -4899,7 +4856,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>arxiv</t>
+          <t>ASE 2023</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5528,7 +5485,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>arxiv</t>
+          <t>Empirical Software Engineering</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -5754,9 +5711,6 @@
 }</t>
         </is>
       </c>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
@@ -6275,7 +6229,6 @@
 }</t>
         </is>
       </c>
-      <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -6361,8 +6314,6 @@
 }</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr">
         <is>
           <t>programming assignments</t>
@@ -7049,7 +7000,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
           <t>-</t>
@@ -7231,8 +7181,6 @@
 }</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr">
         <is>
           <t>vulnerability</t>
@@ -7291,7 +7239,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
           <t>-</t>
@@ -8010,7 +7957,6 @@
 }</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr">
         <is>
           <t>search-based</t>
@@ -8227,7 +8173,6 @@
           <t>ASPLOS</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>['Verilog']</t>
@@ -8259,9 +8204,6 @@
 }</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
@@ -8705,7 +8647,6 @@
 }</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -10496,8 +10437,6 @@
 }</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
       <c r="O118" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -10747,8 +10686,6 @@
 }</t>
         </is>
       </c>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="inlineStr"/>
       <c r="O121" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -11628,7 +11565,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
           <t>-</t>
@@ -11697,7 +11633,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
           <t>-</t>
@@ -12129,7 +12064,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
           <t>-</t>
@@ -13768,8 +13702,6 @@
 }</t>
         </is>
       </c>
-      <c r="M155" t="inlineStr"/>
-      <c r="N155" t="inlineStr"/>
       <c r="O155" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -14807,7 +14739,6 @@
           <t>PLDI</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
           <t>['']</t>
@@ -14839,9 +14770,6 @@
 }</t>
         </is>
       </c>
-      <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
-      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n">
@@ -15145,7 +15073,6 @@
           <t>NIPS</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
           <t>['C', ' C++']</t>
@@ -15196,7 +15123,6 @@
 }</t>
         </is>
       </c>
-      <c r="M171" t="inlineStr"/>
       <c r="N171" t="inlineStr">
         <is>
           <t>learning-based</t>
@@ -15532,7 +15458,6 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L175" t="inlineStr"/>
       <c r="M175" t="inlineStr">
         <is>
           <t>-</t>
@@ -15718,9 +15643,6 @@
 }</t>
         </is>
       </c>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n">
@@ -15749,7 +15671,6 @@
           <t>European Symposium on Research in Computer Security</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
           <t>['Java']</t>
@@ -15799,7 +15720,6 @@
 }</t>
         </is>
       </c>
-      <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr">
         <is>
           <t>search-based</t>
@@ -16393,7 +16313,6 @@
           <t>FSE</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>['']</t>
@@ -16425,8 +16344,6 @@
 }</t>
         </is>
       </c>
-      <c r="M185" t="inlineStr"/>
-      <c r="N185" t="inlineStr"/>
       <c r="O185" t="inlineStr">
         <is>
           <t>programming assignments</t>
@@ -16549,7 +16466,6 @@
           <t>FSE</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
           <t>['']</t>
@@ -16581,8 +16497,6 @@
 }</t>
         </is>
       </c>
-      <c r="M187" t="inlineStr"/>
-      <c r="N187" t="inlineStr"/>
       <c r="O187" t="inlineStr">
         <is>
           <t>programming assignments</t>
@@ -16741,8 +16655,6 @@
 }</t>
         </is>
       </c>
-      <c r="M189" t="inlineStr"/>
-      <c r="N189" t="inlineStr"/>
       <c r="O189" t="inlineStr">
         <is>
           <t>vulnerability</t>
@@ -16812,8 +16724,6 @@
 }</t>
         </is>
       </c>
-      <c r="M190" t="inlineStr"/>
-      <c r="N190" t="inlineStr"/>
       <c r="O190" t="inlineStr">
         <is>
           <t>vulnerabilities</t>
@@ -17422,8 +17332,6 @@
 }</t>
         </is>
       </c>
-      <c r="M197" t="inlineStr"/>
-      <c r="N197" t="inlineStr"/>
       <c r="O197" t="inlineStr">
         <is>
           <t>concurrency bugs</t>
@@ -17590,8 +17498,6 @@
 }</t>
         </is>
       </c>
-      <c r="M199" t="inlineStr"/>
-      <c r="N199" t="inlineStr"/>
       <c r="O199" t="inlineStr">
         <is>
           <t>divide-by-zero and null-dereference errors</t>
@@ -17661,8 +17567,6 @@
 }</t>
         </is>
       </c>
-      <c r="M200" t="inlineStr"/>
-      <c r="N200" t="inlineStr"/>
       <c r="O200" t="inlineStr">
         <is>
           <t>deadlock/livelock</t>
@@ -18118,7 +18022,6 @@
           <t>semantics-based</t>
         </is>
       </c>
-      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n">
@@ -18623,9 +18526,6 @@
           <t>@inproceedings{DBLP:conf/cec/ArcuriY08,   author       = {Andrea Arcuri and                   Xin Yao},   title        = {A novel co-evolutionary approach to automatic software bug fixing},   booktitle    = {Proceedings of the {IEEE} Congress on Evolutionary Computation, {CEC}                   2008, June 1-6, 2008, Hong Kong, China},   pages        = {162--168},   publisher    = {{IEEE}},   year         = {2008},   url          = {https://doi.org/10.1109/CEC.2008.4630793},   doi          = {10.1109/CEC.2008.4630793},   timestamp    = {Thu, 16 Dec 2021 14:01:33 +0100},   biburl       = {https://dblp.org/rec/conf/cec/ArcuriY08.bib},   bibsource    = {dblp computer science bibliography, https://dblp.org} }</t>
         </is>
       </c>
-      <c r="M211" t="inlineStr"/>
-      <c r="N211" t="inlineStr"/>
-      <c r="O211" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: update APR papers (2026-04-01)
</commit_message>
<xml_diff>
--- a/metadata_manager/output/apr_literature_metadata.xlsx
+++ b/metadata_manager/output/apr_literature_metadata.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,84 +417,84 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>APR Tool Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Venue</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Repo URL</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Target Language</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Used Dataset</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>CCF Rank</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Paper Category</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Bibtex</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Specification</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Tool Category</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Bug Types</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -549,7 +537,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>B</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -579,7 +567,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -632,7 +620,7 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -701,7 +689,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -775,7 +763,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -844,7 +832,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -922,7 +910,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -1003,7 +991,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -1066,7 +1054,7 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -1124,7 +1112,7 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -1197,7 +1185,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -1263,7 +1251,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1337,7 +1325,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1430,7 +1418,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1512,7 +1500,7 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1591,7 +1579,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1677,7 +1665,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1771,7 +1759,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>17</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1859,7 +1847,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>18</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1947,7 +1935,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>19</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -2028,7 +2016,7 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>20</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -2120,7 +2108,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -2193,7 +2181,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -2271,7 +2259,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -2347,7 +2335,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>24</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -2431,7 +2419,7 @@
       <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -2490,7 +2478,7 @@
       <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>26</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -2600,7 +2588,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>27</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -2694,7 +2682,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>28</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -2786,7 +2774,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>29</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -2879,7 +2867,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>30</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -2968,7 +2956,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>31</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -3055,7 +3043,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>32</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -3146,7 +3134,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>33</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -3237,7 +3225,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>34</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -3318,7 +3306,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>35</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -3376,7 +3364,7 @@
       <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>36</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -3449,7 +3437,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>37</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -3528,7 +3516,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>38</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -3607,7 +3595,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>39</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -3698,7 +3686,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>40</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -3775,7 +3763,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>41</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -3854,7 +3842,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>42</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -3956,7 +3944,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>43</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -4040,7 +4028,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>44</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -4119,7 +4107,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>45</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -4192,7 +4180,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>46</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -4284,7 +4272,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" t="n">
         <v>47</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -4365,7 +4353,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" t="n">
         <v>48</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -4455,7 +4443,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" t="n">
         <v>49</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -4541,7 +4529,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" t="n">
         <v>50</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -4630,7 +4618,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" t="n">
         <v>51</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -4724,7 +4712,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" t="n">
         <v>52</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -4815,7 +4803,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" t="n">
         <v>53</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -4900,7 +4888,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" t="n">
         <v>54</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -4973,7 +4961,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" t="n">
         <v>55</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -5062,7 +5050,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" t="n">
         <v>56</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -5155,7 +5143,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" t="n">
         <v>57</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -5243,7 +5231,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" t="n">
         <v>58</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -5335,7 +5323,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" t="n">
         <v>59</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -5427,7 +5415,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" t="n">
         <v>60</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -5515,7 +5503,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" t="n">
         <v>61</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -5603,7 +5591,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" t="n">
         <v>62</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -5679,7 +5667,7 @@
       <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" t="n">
         <v>63</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -5772,7 +5760,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" t="n">
         <v>64</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -5859,7 +5847,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" t="n">
         <v>65</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -5949,7 +5937,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" t="n">
         <v>66</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -6028,7 +6016,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" t="n">
         <v>67</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -6118,7 +6106,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" t="n">
         <v>68</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -6208,7 +6196,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" t="n">
         <v>69</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -6290,7 +6278,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" t="n">
         <v>70</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -6378,7 +6366,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" t="n">
         <v>71</v>
       </c>
       <c r="B73" t="inlineStr">
@@ -6471,7 +6459,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" t="n">
         <v>72</v>
       </c>
       <c r="B74" t="inlineStr">
@@ -6560,7 +6548,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" t="n">
         <v>73</v>
       </c>
       <c r="B75" t="inlineStr">
@@ -6646,7 +6634,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" t="n">
         <v>74</v>
       </c>
       <c r="B76" t="inlineStr">
@@ -6736,7 +6724,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" t="n">
         <v>75</v>
       </c>
       <c r="B77" t="inlineStr">
@@ -6826,7 +6814,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" t="n">
         <v>76</v>
       </c>
       <c r="B78" t="inlineStr">
@@ -6918,7 +6906,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" t="n">
         <v>77</v>
       </c>
       <c r="B79" t="inlineStr">
@@ -6987,7 +6975,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" t="n">
         <v>78</v>
       </c>
       <c r="B80" t="inlineStr">
@@ -7077,7 +7065,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" t="n">
         <v>79</v>
       </c>
       <c r="B81" t="inlineStr">
@@ -7160,7 +7148,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" t="n">
         <v>80</v>
       </c>
       <c r="B82" t="inlineStr">
@@ -7229,7 +7217,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" t="n">
         <v>81</v>
       </c>
       <c r="B83" t="inlineStr">
@@ -7322,7 +7310,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" t="n">
         <v>82</v>
       </c>
       <c r="B84" t="inlineStr">
@@ -7410,7 +7398,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" t="n">
         <v>83</v>
       </c>
       <c r="B85" t="inlineStr">
@@ -7502,7 +7490,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" t="n">
         <v>84</v>
       </c>
       <c r="B86" t="inlineStr">
@@ -7596,7 +7584,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" t="n">
         <v>85</v>
       </c>
       <c r="B87" t="inlineStr">
@@ -7687,7 +7675,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" t="n">
         <v>86</v>
       </c>
       <c r="B88" t="inlineStr">
@@ -7776,7 +7764,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" t="n">
         <v>87</v>
       </c>
       <c r="B89" t="inlineStr">
@@ -7868,7 +7856,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" t="n">
         <v>88</v>
       </c>
       <c r="B90" t="inlineStr">
@@ -7943,7 +7931,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" t="n">
         <v>89</v>
       </c>
       <c r="B91" t="inlineStr">
@@ -8032,7 +8020,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" t="n">
         <v>90</v>
       </c>
       <c r="B92" t="inlineStr">
@@ -8121,7 +8109,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
+      <c r="A93" t="n">
         <v>91</v>
       </c>
       <c r="B93" t="inlineStr">
@@ -8184,7 +8172,7 @@
       <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
+      <c r="A94" t="n">
         <v>92</v>
       </c>
       <c r="B94" t="inlineStr">
@@ -8273,7 +8261,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
+      <c r="A95" t="n">
         <v>93</v>
       </c>
       <c r="B95" t="inlineStr">
@@ -8361,7 +8349,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
+      <c r="A96" t="n">
         <v>94</v>
       </c>
       <c r="B96" t="inlineStr">
@@ -8455,7 +8443,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
+      <c r="A97" t="n">
         <v>95</v>
       </c>
       <c r="B97" t="inlineStr">
@@ -8550,7 +8538,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
+      <c r="A98" t="n">
         <v>96</v>
       </c>
       <c r="B98" t="inlineStr">
@@ -8638,7 +8626,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
+      <c r="A99" t="n">
         <v>97</v>
       </c>
       <c r="B99" t="inlineStr">
@@ -8728,7 +8716,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
+      <c r="A100" t="n">
         <v>98</v>
       </c>
       <c r="B100" t="inlineStr">
@@ -8818,7 +8806,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
+      <c r="A101" t="n">
         <v>99</v>
       </c>
       <c r="B101" t="inlineStr">
@@ -8909,7 +8897,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
+      <c r="A102" t="n">
         <v>100</v>
       </c>
       <c r="B102" t="inlineStr">
@@ -9001,7 +8989,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
+      <c r="A103" t="n">
         <v>101</v>
       </c>
       <c r="B103" t="inlineStr">
@@ -9091,7 +9079,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
+      <c r="A104" t="n">
         <v>102</v>
       </c>
       <c r="B104" t="inlineStr">
@@ -9179,7 +9167,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
+      <c r="A105" t="n">
         <v>103</v>
       </c>
       <c r="B105" t="inlineStr">
@@ -9274,7 +9262,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
+      <c r="A106" t="n">
         <v>104</v>
       </c>
       <c r="B106" t="inlineStr">
@@ -9361,7 +9349,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
+      <c r="A107" t="n">
         <v>105</v>
       </c>
       <c r="B107" t="inlineStr">
@@ -9450,7 +9438,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
+      <c r="A108" t="n">
         <v>106</v>
       </c>
       <c r="B108" t="inlineStr">
@@ -9540,7 +9528,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
+      <c r="A109" t="n">
         <v>107</v>
       </c>
       <c r="B109" t="inlineStr">
@@ -9632,7 +9620,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
+      <c r="A110" t="n">
         <v>108</v>
       </c>
       <c r="B110" t="inlineStr">
@@ -9723,7 +9711,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
+      <c r="A111" t="n">
         <v>109</v>
       </c>
       <c r="B111" t="inlineStr">
@@ -9816,7 +9804,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
+      <c r="A112" t="n">
         <v>110</v>
       </c>
       <c r="B112" t="inlineStr">
@@ -9911,7 +9899,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
+      <c r="A113" t="n">
         <v>111</v>
       </c>
       <c r="B113" t="inlineStr">
@@ -9999,7 +9987,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
+      <c r="A114" t="n">
         <v>112</v>
       </c>
       <c r="B114" t="inlineStr">
@@ -10088,7 +10076,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
+      <c r="A115" t="n">
         <v>113</v>
       </c>
       <c r="B115" t="inlineStr">
@@ -10179,7 +10167,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
+      <c r="A116" t="n">
         <v>114</v>
       </c>
       <c r="B116" t="inlineStr">
@@ -10267,7 +10255,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
+      <c r="A117" t="n">
         <v>115</v>
       </c>
       <c r="B117" t="inlineStr">
@@ -10355,7 +10343,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
+      <c r="A118" t="n">
         <v>116</v>
       </c>
       <c r="B118" t="inlineStr">
@@ -10425,7 +10413,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
+      <c r="A119" t="n">
         <v>117</v>
       </c>
       <c r="B119" t="inlineStr">
@@ -10514,7 +10502,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
+      <c r="A120" t="n">
         <v>118</v>
       </c>
       <c r="B120" t="inlineStr">
@@ -10602,7 +10590,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
+      <c r="A121" t="n">
         <v>119</v>
       </c>
       <c r="B121" t="inlineStr">
@@ -10676,7 +10664,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
+      <c r="A122" t="n">
         <v>120</v>
       </c>
       <c r="B122" t="inlineStr">
@@ -10767,7 +10755,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
+      <c r="A123" t="n">
         <v>121</v>
       </c>
       <c r="B123" t="inlineStr">
@@ -10862,7 +10850,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
+      <c r="A124" t="n">
         <v>122</v>
       </c>
       <c r="B124" t="inlineStr">
@@ -10949,7 +10937,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
+      <c r="A125" t="n">
         <v>123</v>
       </c>
       <c r="B125" t="inlineStr">
@@ -11036,7 +11024,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
+      <c r="A126" t="n">
         <v>124</v>
       </c>
       <c r="B126" t="inlineStr">
@@ -11128,7 +11116,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
+      <c r="A127" t="n">
         <v>125</v>
       </c>
       <c r="B127" t="inlineStr">
@@ -11225,7 +11213,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
+      <c r="A128" t="n">
         <v>126</v>
       </c>
       <c r="B128" t="inlineStr">
@@ -11321,7 +11309,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
+      <c r="A129" t="n">
         <v>127</v>
       </c>
       <c r="B129" t="inlineStr">
@@ -11408,7 +11396,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
+      <c r="A130" t="n">
         <v>128</v>
       </c>
       <c r="B130" t="inlineStr">
@@ -11497,7 +11485,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
+      <c r="A131" t="n">
         <v>129</v>
       </c>
       <c r="B131" t="inlineStr">
@@ -11566,7 +11554,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
+      <c r="A132" t="n">
         <v>130</v>
       </c>
       <c r="B132" t="inlineStr">
@@ -11635,7 +11623,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
+      <c r="A133" t="n">
         <v>131</v>
       </c>
       <c r="B133" t="inlineStr">
@@ -11727,7 +11715,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
+      <c r="A134" t="n">
         <v>132</v>
       </c>
       <c r="B134" t="inlineStr">
@@ -11818,7 +11806,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
+      <c r="A135" t="n">
         <v>133</v>
       </c>
       <c r="B135" t="inlineStr">
@@ -11912,7 +11900,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
+      <c r="A136" t="n">
         <v>134</v>
       </c>
       <c r="B136" t="inlineStr">
@@ -11998,7 +11986,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
+      <c r="A137" t="n">
         <v>135</v>
       </c>
       <c r="B137" t="inlineStr">
@@ -12067,7 +12055,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
+      <c r="A138" t="n">
         <v>136</v>
       </c>
       <c r="B138" t="inlineStr">
@@ -12160,7 +12148,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="1" t="n">
+      <c r="A139" t="n">
         <v>137</v>
       </c>
       <c r="B139" t="inlineStr">
@@ -12248,7 +12236,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="1" t="n">
+      <c r="A140" t="n">
         <v>138</v>
       </c>
       <c r="B140" t="inlineStr">
@@ -12345,7 +12333,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="1" t="n">
+      <c r="A141" t="n">
         <v>139</v>
       </c>
       <c r="B141" t="inlineStr">
@@ -12437,7 +12425,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="1" t="n">
+      <c r="A142" t="n">
         <v>140</v>
       </c>
       <c r="B142" t="inlineStr">
@@ -12529,7 +12517,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="1" t="n">
+      <c r="A143" t="n">
         <v>141</v>
       </c>
       <c r="B143" t="inlineStr">
@@ -12621,7 +12609,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="1" t="n">
+      <c r="A144" t="n">
         <v>142</v>
       </c>
       <c r="B144" t="inlineStr">
@@ -12714,7 +12702,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="1" t="n">
+      <c r="A145" t="n">
         <v>143</v>
       </c>
       <c r="B145" t="inlineStr">
@@ -12809,7 +12797,7 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="1" t="n">
+      <c r="A146" t="n">
         <v>144</v>
       </c>
       <c r="B146" t="inlineStr">
@@ -12899,7 +12887,7 @@
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="1" t="n">
+      <c r="A147" t="n">
         <v>145</v>
       </c>
       <c r="B147" t="inlineStr">
@@ -12987,7 +12975,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="1" t="n">
+      <c r="A148" t="n">
         <v>146</v>
       </c>
       <c r="B148" t="inlineStr">
@@ -13078,7 +13066,7 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="1" t="n">
+      <c r="A149" t="n">
         <v>147</v>
       </c>
       <c r="B149" t="inlineStr">
@@ -13167,7 +13155,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="1" t="n">
+      <c r="A150" t="n">
         <v>148</v>
       </c>
       <c r="B150" t="inlineStr">
@@ -13261,7 +13249,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="1" t="n">
+      <c r="A151" t="n">
         <v>149</v>
       </c>
       <c r="B151" t="inlineStr">
@@ -13350,7 +13338,7 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="1" t="n">
+      <c r="A152" t="n">
         <v>150</v>
       </c>
       <c r="B152" t="inlineStr">
@@ -13445,7 +13433,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="1" t="n">
+      <c r="A153" t="n">
         <v>151</v>
       </c>
       <c r="B153" t="inlineStr">
@@ -13536,7 +13524,7 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="1" t="n">
+      <c r="A154" t="n">
         <v>152</v>
       </c>
       <c r="B154" t="inlineStr">
@@ -13626,7 +13614,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="1" t="n">
+      <c r="A155" t="n">
         <v>153</v>
       </c>
       <c r="B155" t="inlineStr">
@@ -13697,7 +13685,7 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="1" t="n">
+      <c r="A156" t="n">
         <v>154</v>
       </c>
       <c r="B156" t="inlineStr">
@@ -13786,7 +13774,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="1" t="n">
+      <c r="A157" t="n">
         <v>155</v>
       </c>
       <c r="B157" t="inlineStr">
@@ -13877,7 +13865,7 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="1" t="n">
+      <c r="A158" t="n">
         <v>156</v>
       </c>
       <c r="B158" t="inlineStr">
@@ -13971,7 +13959,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="1" t="n">
+      <c r="A159" t="n">
         <v>157</v>
       </c>
       <c r="B159" t="inlineStr">
@@ -14058,7 +14046,7 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="1" t="n">
+      <c r="A160" t="n">
         <v>158</v>
       </c>
       <c r="B160" t="inlineStr">
@@ -14152,7 +14140,7 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="1" t="n">
+      <c r="A161" t="n">
         <v>159</v>
       </c>
       <c r="B161" t="inlineStr">
@@ -14244,7 +14232,7 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="1" t="n">
+      <c r="A162" t="n">
         <v>160</v>
       </c>
       <c r="B162" t="inlineStr">
@@ -14337,7 +14325,7 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="1" t="n">
+      <c r="A163" t="n">
         <v>161</v>
       </c>
       <c r="B163" t="inlineStr">
@@ -14423,7 +14411,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="1" t="n">
+      <c r="A164" t="n">
         <v>162</v>
       </c>
       <c r="B164" t="inlineStr">
@@ -14514,7 +14502,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="1" t="n">
+      <c r="A165" t="n">
         <v>163</v>
       </c>
       <c r="B165" t="inlineStr">
@@ -14607,7 +14595,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="1" t="n">
+      <c r="A166" t="n">
         <v>164</v>
       </c>
       <c r="B166" t="inlineStr">
@@ -14701,7 +14689,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="1" t="n">
+      <c r="A167" t="n">
         <v>165</v>
       </c>
       <c r="B167" t="inlineStr">
@@ -14764,7 +14752,7 @@
       <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" s="1" t="n">
+      <c r="A168" t="n">
         <v>166</v>
       </c>
       <c r="B168" t="inlineStr">
@@ -14857,7 +14845,7 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="1" t="n">
+      <c r="A169" t="n">
         <v>167</v>
       </c>
       <c r="B169" t="inlineStr">
@@ -14949,7 +14937,7 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="1" t="n">
+      <c r="A170" t="n">
         <v>168</v>
       </c>
       <c r="B170" t="inlineStr">
@@ -15039,7 +15027,7 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="1" t="n">
+      <c r="A171" t="n">
         <v>169</v>
       </c>
       <c r="B171" t="inlineStr">
@@ -15129,7 +15117,7 @@
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="1" t="n">
+      <c r="A172" t="n">
         <v>170</v>
       </c>
       <c r="B172" t="inlineStr">
@@ -15219,7 +15207,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="1" t="n">
+      <c r="A173" t="n">
         <v>171</v>
       </c>
       <c r="B173" t="inlineStr">
@@ -15307,7 +15295,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="1" t="n">
+      <c r="A174" t="n">
         <v>172</v>
       </c>
       <c r="B174" t="inlineStr">
@@ -15401,7 +15389,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="1" t="n">
+      <c r="A175" t="n">
         <v>173</v>
       </c>
       <c r="B175" t="inlineStr">
@@ -15470,7 +15458,7 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="1" t="n">
+      <c r="A176" t="n">
         <v>174</v>
       </c>
       <c r="B176" t="inlineStr">
@@ -15563,7 +15551,7 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="1" t="n">
+      <c r="A177" t="n">
         <v>175</v>
       </c>
       <c r="B177" t="inlineStr">
@@ -15643,7 +15631,7 @@
       <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="1" t="n">
+      <c r="A178" t="n">
         <v>176</v>
       </c>
       <c r="B178" t="inlineStr">
@@ -15732,7 +15720,7 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="1" t="n">
+      <c r="A179" t="n">
         <v>177</v>
       </c>
       <c r="B179" t="inlineStr">
@@ -15823,7 +15811,7 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="1" t="n">
+      <c r="A180" t="n">
         <v>178</v>
       </c>
       <c r="B180" t="inlineStr">
@@ -15919,7 +15907,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="1" t="n">
+      <c r="A181" t="n">
         <v>179</v>
       </c>
       <c r="B181" t="inlineStr">
@@ -16014,7 +16002,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="1" t="n">
+      <c r="A182" t="n">
         <v>180</v>
       </c>
       <c r="B182" t="inlineStr">
@@ -16105,7 +16093,7 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="1" t="n">
+      <c r="A183" t="n">
         <v>181</v>
       </c>
       <c r="B183" t="inlineStr">
@@ -16195,7 +16183,7 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="1" t="n">
+      <c r="A184" t="n">
         <v>182</v>
       </c>
       <c r="B184" t="inlineStr">
@@ -16287,7 +16275,7 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="1" t="n">
+      <c r="A185" t="n">
         <v>183</v>
       </c>
       <c r="B185" t="inlineStr">
@@ -16354,7 +16342,7 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="1" t="n">
+      <c r="A186" t="n">
         <v>184</v>
       </c>
       <c r="B186" t="inlineStr">
@@ -16443,7 +16431,7 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="1" t="n">
+      <c r="A187" t="n">
         <v>185</v>
       </c>
       <c r="B187" t="inlineStr">
@@ -16510,7 +16498,7 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="1" t="n">
+      <c r="A188" t="n">
         <v>186</v>
       </c>
       <c r="B188" t="inlineStr">
@@ -16599,7 +16587,7 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="1" t="n">
+      <c r="A189" t="n">
         <v>187</v>
       </c>
       <c r="B189" t="inlineStr">
@@ -16670,7 +16658,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="1" t="n">
+      <c r="A190" t="n">
         <v>188</v>
       </c>
       <c r="B190" t="inlineStr">
@@ -16741,7 +16729,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="1" t="n">
+      <c r="A191" t="n">
         <v>189</v>
       </c>
       <c r="B191" t="inlineStr">
@@ -16829,7 +16817,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="1" t="n">
+      <c r="A192" t="n">
         <v>190</v>
       </c>
       <c r="B192" t="inlineStr">
@@ -16919,7 +16907,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="1" t="n">
+      <c r="A193" t="n">
         <v>191</v>
       </c>
       <c r="B193" t="inlineStr">
@@ -17010,7 +16998,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="1" t="n">
+      <c r="A194" t="n">
         <v>192</v>
       </c>
       <c r="B194" t="inlineStr">
@@ -17101,7 +17089,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="1" t="n">
+      <c r="A195" t="n">
         <v>193</v>
       </c>
       <c r="B195" t="inlineStr">
@@ -17189,7 +17177,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="1" t="n">
+      <c r="A196" t="n">
         <v>194</v>
       </c>
       <c r="B196" t="inlineStr">
@@ -17280,7 +17268,7 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="1" t="n">
+      <c r="A197" t="n">
         <v>195</v>
       </c>
       <c r="B197" t="inlineStr">
@@ -17351,7 +17339,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="1" t="n">
+      <c r="A198" t="n">
         <v>196</v>
       </c>
       <c r="B198" t="inlineStr">
@@ -17437,7 +17425,7 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="1" t="n">
+      <c r="A199" t="n">
         <v>197</v>
       </c>
       <c r="B199" t="inlineStr">
@@ -17519,7 +17507,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="1" t="n">
+      <c r="A200" t="n">
         <v>198</v>
       </c>
       <c r="B200" t="inlineStr">
@@ -17590,7 +17578,7 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="1" t="n">
+      <c r="A201" t="n">
         <v>199</v>
       </c>
       <c r="B201" t="inlineStr">
@@ -17681,7 +17669,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="1" t="n">
+      <c r="A202" t="n">
         <v>200</v>
       </c>
       <c r="B202" t="inlineStr">
@@ -17772,7 +17760,7 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="1" t="n">
+      <c r="A203" t="n">
         <v>201</v>
       </c>
       <c r="B203" t="inlineStr">
@@ -17860,7 +17848,7 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="1" t="n">
+      <c r="A204" t="n">
         <v>202</v>
       </c>
       <c r="B204" t="inlineStr">
@@ -17952,7 +17940,7 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="1" t="n">
+      <c r="A205" t="n">
         <v>203</v>
       </c>
       <c r="B205" t="inlineStr">
@@ -18041,7 +18029,7 @@
       <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
-      <c r="A206" s="1" t="n">
+      <c r="A206" t="n">
         <v>204</v>
       </c>
       <c r="B206" t="inlineStr">
@@ -18127,7 +18115,7 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="1" t="n">
+      <c r="A207" t="n">
         <v>205</v>
       </c>
       <c r="B207" t="inlineStr">
@@ -18220,7 +18208,7 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="1" t="n">
+      <c r="A208" t="n">
         <v>206</v>
       </c>
       <c r="B208" t="inlineStr">
@@ -18310,7 +18298,7 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="1" t="n">
+      <c r="A209" t="n">
         <v>207</v>
       </c>
       <c r="B209" t="inlineStr">
@@ -18398,7 +18386,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="1" t="n">
+      <c r="A210" t="n">
         <v>208</v>
       </c>
       <c r="B210" t="inlineStr">
@@ -18487,7 +18475,7 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="1" t="n">
+      <c r="A211" t="n">
         <v>209</v>
       </c>
       <c r="B211" t="inlineStr">

</xml_diff>